<commit_message>
Updated classes to relationship and updated message to align with CORE-000229 and CORE-000230
</commit_message>
<xml_diff>
--- a/rules/CORE-000231/negative/01/data/unit-test-coreid-CG0363-negative.xlsx
+++ b/rules/CORE-000231/negative/01/data/unit-test-coreid-CG0363-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -53,6 +53,15 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <i/>
     </font>
     <font>
@@ -64,7 +73,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -72,6 +81,12 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -113,15 +128,16 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,11 +480,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
-        <v>3-2</v>
+      <c r="B2" s="4" t="str">
+        <v>3-3</v>
       </c>
     </row>
   </sheetData>
@@ -491,10 +507,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>relsub.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Related Subjects</v>
       </c>
     </row>
@@ -530,82 +546,82 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>relsub.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>RSUBJID</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v>HEM021-001</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>relsub.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>5</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="4" t="str">
         <v>USUBJID</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="4" t="str">
         <v>HEM021-001</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="str">
+      <c r="B4" s="4" t="str">
         <v>relsub.xpt</v>
       </c>
-      <c r="C4" s="2" t="str">
+      <c r="C4" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <v>8</v>
       </c>
-      <c r="E4" s="2" t="str">
+      <c r="E4" s="4" t="str">
         <v>RSUBJID</v>
       </c>
-      <c r="F4" s="2" t="str">
+      <c r="F4" s="4" t="str">
         <v>HEM021-004</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
+      <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="str">
+      <c r="B5" s="4" t="str">
         <v>relsub.xpt</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="4">
         <v>8</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="4" t="str">
         <v>USUBJID</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="4" t="str">
         <v>HEM021-004</v>
       </c>
     </row>
@@ -638,121 +654,121 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="C2" s="4" t="str">
+      <c r="C2" s="6" t="str">
         <v>Pool Identifier</v>
       </c>
-      <c r="D2" s="4" t="str">
+      <c r="D2" s="6" t="str">
         <v>Related Subject or Pool Identifier</v>
       </c>
-      <c r="E2" s="4" t="str">
+      <c r="E2" s="6" t="str">
         <v>Subject Relationship</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="str">
+      <c r="A3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="4" t="str">
+      <c r="B3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="4" t="str">
+      <c r="C3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="4" t="str">
+      <c r="D3" s="6" t="str">
         <v>Char</v>
       </c>
-      <c r="E3" s="4" t="str">
+      <c r="E3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="6">
         <v>50</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="6">
         <v>50</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="6">
         <v>50</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="6">
         <v>50</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="6">
         <v>50</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="str">
+      <c r="A5" s="4" t="str">
         <v>HEM021</v>
       </c>
-      <c r="B5" s="5" t="str">
+      <c r="B5" s="7" t="str">
         <v>HEM021-001</v>
       </c>
-      <c r="C5" s="2" t="str">
+      <c r="C5" s="4" t="str">
         <v>HEM021-001</v>
       </c>
-      <c r="D5" s="6" t="str">
+      <c r="D5" s="8" t="str">
         <v>HEM021-001</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="4" t="str">
         <v>MOTHER,BIOLOGICAL</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="str">
+      <c r="A6" s="4" t="str">
         <v>HEM021</v>
       </c>
-      <c r="B6" s="2" t="str">
+      <c r="B6" s="4" t="str">
         <v>HEM021-002</v>
       </c>
-      <c r="C6" s="2" t="str">
+      <c r="C6" s="4" t="str">
         <v>HEM021-001</v>
       </c>
-      <c r="D6" s="7" t="str">
+      <c r="D6" s="4" t="str">
         <v>Hem021-002</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E6" s="4" t="str">
         <v>MOTHER,BIOLOGICAL</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="str">
+      <c r="A7" s="4" t="str">
         <v>HEM021</v>
       </c>
-      <c r="B7" s="2" t="str">
+      <c r="B7" s="4" t="str">
         <v>Hem021-003</v>
       </c>
-      <c r="C7" s="2" t="str">
+      <c r="C7" s="4" t="str">
         <v>HEM021-002</v>
       </c>
-      <c r="D7" s="7" t="str">
+      <c r="D7" s="4" t="str">
         <v>HEM021-003</v>
       </c>
-      <c r="E7" s="2" t="str">
+      <c r="E7" s="4" t="str">
         <v>CHILD, BIOLOGICAL</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="str">
+      <c r="A8" s="4" t="str">
         <v>HEM021</v>
       </c>
-      <c r="B8" s="5" t="str">
+      <c r="B8" s="8" t="str">
         <v>HEM021-004</v>
       </c>
-      <c r="C8" s="2" t="str">
+      <c r="C8" s="4" t="str">
         <v>HEM021-002</v>
       </c>
-      <c r="D8" s="6" t="str">
+      <c r="D8" s="8" t="str">
         <v>HEM021-004</v>
       </c>
-      <c r="E8" s="2" t="str">
+      <c r="E8" s="4" t="str">
         <v>TWIN,DIZYGOTIC</v>
       </c>
     </row>

</xml_diff>